<commit_message>
feat(P-2026-0044): incorporar desmontaje y montaje de tabica (186,50 m2) y falso techo inferior (533,60 m2) a REV5
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto-cliente.xlsx
+++ b/presupuestos/P-2026-0044-sustitucion-cubierta-terminal-carga-aeropuerto-menorca/presupuesto-cliente.xlsx
@@ -31,21 +31,23 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000F172A"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00B91C1C"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="000F172A"/>
       <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
+      <color rgb="001E293B"/>
       <sz val="9.5"/>
     </font>
     <font>
@@ -63,19 +65,19 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="10"/>
+      <color rgb="00B91C1C"/>
+      <sz val="10.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="11.5"/>
+      <color rgb="00065F46"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0015803D"/>
+      <color rgb="00B91C1C"/>
       <sz val="12"/>
     </font>
     <font>
@@ -106,8 +108,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00E2E8F0"/>
+        <bgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -124,8 +126,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-        <bgColor rgb="00FEF2F2"/>
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -142,8 +144,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00FEF2F2"/>
+        <bgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -183,7 +185,7 @@
     </border>
     <border>
       <top style="thin">
-        <color rgb="000F172A"/>
+        <color rgb="00CBD5E1"/>
       </top>
       <bottom style="double">
         <color rgb="000F172A"/>
@@ -245,10 +247,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -259,14 +261,14 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -667,28 +669,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HAM ESTRUCTURAS METÁLICAS</t>
+          <t>HAM ESTRUCTURAS METÁLICAS (DIXIS RECURSOS Y SOLUCIONES, SL)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0044</t>
+          <t>PRESUPUESTO TÉCNICO OFICIAL: P-2026-0044 | REF: PRE-2026-1028-AENA-CARGA-HDX-REV5</t>
         </is>
       </c>
     </row>
@@ -700,7 +702,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Consultores de Ingeniería UG21 / UTE BTG-UG21 (Atn: Marina Gallego Fernández (Arquitecto / Proyectos))</t>
+          <t>Consultores de Ingeniería UG21 / UTE BTG-UG21 | Atn: Marina Gallego Fernández (Arquitecto / Proyectos)</t>
         </is>
       </c>
     </row>
@@ -712,31 +714,31 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>100.174 Sustitución Cubierta Terminal de Carga - Proyecto Básico - Promotor: AENA S.M.E., S.A. - Dirección de Infraestructuras</t>
+          <t>100.174 Sustitución Cubierta Terminal de Carga - Proyecto Básico | Promotor: AENA S.M.E., S.A. - Dirección de Infraestructuras</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Ubicación:</t>
+          <t>Emplazamiento:</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Terminal de Carga, Aeropuerto de Menorca, Carretera de Sant Climent, s/n, 07712 Mahón (Menorca)</t>
+          <t>Terminal de Carga, Aeropuerto de Menorca, Mahón (Menorca)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Fecha:</t>
+          <t>Fecha de emisión:</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
     </row>
@@ -748,7 +750,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) con acabado Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones roscachapa galvanizadas con arandela vulcanizada EPDM | Medios mecánicos y fletes integrados | Opcionales: 2 escalas de gato inox con crinolina (+30%) + Línea LuxTop® (18.000 €)</t>
+          <t>Panel Sándwich Cubierta PIR 40 mm (B-s1,d0) + Chapas grecadas voladizos y tabica con acabado Granite® HDX55 (55 µm) por AMBAS CARAS | Fijaciones roscachapa galvanizadas con arandela vulcanizada EPDM | Medios mecánicos y fletes integrados | Opcionales: 2 escalas de gato inox con crinolina (+30%) + Línea LuxTop® (18.000 €)</t>
         </is>
       </c>
     </row>
@@ -859,7 +861,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Voladizos en fachadas (muelles de carga)</t>
+          <t>Voladizos en fachadas (cobertura superior)</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -882,506 +884,567 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr"/>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Lado inferior de voladizos (cielo raso)</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Chapa grecada bajo viguetas en ménsula</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>533.6</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Granite® HDX55 (2 caras)</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Marino C5-M / Aéreo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Tabica vertical de fachada sobre marquesinas</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Chapa grecada en paramento vertical</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>186.5</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Granite® HDX55 (2 caras)</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Marino C5-M / Aéreo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr"/>
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>TOTAL SUPERFICIE DE ACTUACIÓN:</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr"/>
-      <c r="D16" s="14">
-        <f>SUM(D13:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr"/>
+      <c r="D18" s="14">
+        <f>SUM(D13:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>m² totales</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>VALORACIÓN ECONÓMICA DE PARTIDAS BASE (CON MEDIOS INTEGRADOS)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Partida</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Concepto y Descripción Técnica</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>Precio Unitario (€)</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>Importe (€)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Desmontaje controlado de cubierta actual, voladizos existentes y gestión autorizada de residuos
-Desmontaje manual y mecánico de la cubierta y voladizos existentes de chapa/panel degradada y corroída. Incluye descenso a cota cero con grúa pluma y plataforma elevadora (medios integrados), acopio, clasificación de residuos férricos, carga, transporte y entrega en centro autorizado de gestión y reciclaje de residuos de Menorca, con tasas y canon oficial de vertedero incluidos.</t>
-        </is>
-      </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Desmontaje controlado de cubierta actual, voladizos, falso techo inferior, tabicas y gestión autorizada de residuos
+Desmontaje manual y mecánico de la totalidad de la cubierta existente, chapas de voladizos superiores, falsos techos inferiores de viguetas y tabicas verticales degradadas y corroídas (superficie total 2.624,10 m²). Incluye descenso a cota cero con grúa pluma y plataforma elevadora (medios integrados), acopio clasificado de chatarra férrica, carga, transporte y entrega en centro autorizado de reciclaje de Menorca con canon oficial de vertedero incluido.</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D20" s="19" t="n">
-        <v>1904</v>
-      </c>
-      <c r="E20" s="20" t="n">
+      <c r="D22" s="19" t="n">
+        <v>2624.1</v>
+      </c>
+      <c r="E22" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="F20" s="20">
-        <f>D20*E20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="F22" s="20">
+        <f>D22*E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>Suministro e instalación de Panel Sándwich HDX55 en AMBAS CARAS en cubierta a dos aguas
 Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado, compuesto por núcleo aislante rígido de PIR de 40 mm de espesor (densidad 40 kg/m³, λ = 0,022 W/m·K, clasificación al fuego B-s1,d0) y dos chapas de acero estructural galvanizado con revestimiento de protección marina severa Granite® HDX55 (55 µm de espesor) en AMBAS CARAS (exterior e interior). Fijación a estructura portante mediante tornillería roscachapa / autorroscante de acero galvanizado con arandela estanca vulcanizada de EPDM y cordón continuo de masilla hidro-expansiva de butilo en solapes. Incluye fletes marítimos Península-Menorca de paneles de gran longitud, camión grúa pluma para descarga e izado distribuido en pórticos y plataformas elevadoras PEMP integradas.</t>
         </is>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D23" s="19" t="n">
         <v>1042.5</v>
       </c>
-      <c r="E21" s="20" t="n">
+      <c r="E23" s="20" t="n">
         <v>135</v>
       </c>
-      <c r="F21" s="20">
-        <f>D21*E21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="F23" s="20">
+        <f>D23*E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Suministro e instalación de Panel Sándwich HDX55 en AMBAS CARAS en cubierta a un agua
 Suministro e instalación de panel sándwich de cubierta de 3 grecas con tapajuntas integrado (espesor 40 mm PIR, B-s1,d0) con acabado de alta durabilidad Granite® HDX55 (55 µm) por ambas caras (exterior e interior) en faldón a un agua. Incluye adaptaciones mecánicas de faldón, cortes en encuentros contra paramentos verticales y petos, fijaciones roscachapa de acero galvanizado con arandela de estanqueidad EPDM, sellado butílico continuo y repercusión íntegra de fletes marítimos y medios mecánicos de elevación y PEMP.</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D24" s="19" t="n">
         <v>328.5</v>
       </c>
-      <c r="E22" s="20" t="n">
+      <c r="E24" s="20" t="n">
         <v>135</v>
       </c>
-      <c r="F22" s="20">
-        <f>D22*E22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="F24" s="20">
+        <f>D24*E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Sustitución integral de voladizos en muelles de carga con acabado HDX55 e imprimación anticorrosiva
-Rehabilitación y sustitución completa de la envolvente de los voladizos de fachada (muelles de carga, 267 m² por fachada, total 533 m²). Incluye cepillado y saneado mecánico superficial con eliminación de óxido en viguetas metálicas en ménsula existentes, aplicación de capa de imprimación epoxi anticorrosiva rica en zinc de alto espesor (C5-M), e instalación de nueva cobertura con chapa/panel de alta resistencia protegida con revestimiento HDX55 (55 µm) en ambas caras, con tornillería roscachapa galvanizada con arandela EPDM, remates perimetrales frontales con goterón y repercusión de plataformas elevadoras PEMP.</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Sustitución de cobertura superior de voladizos en muelles de carga con acabado HDX55 e imprimación anticorrosiva
+Rehabilitación y sustitución de la cubierta superior de los voladizos de fachada (muelles de carga, 267 m² por fachada, total 533 m²). Incluye cepillado y saneado mecánico superficial con eliminación de óxido en viguetas metálicas en ménsula existentes, aplicación de capa de imprimación epoxi anticorrosiva rica en zinc de alto espesor (C5-M), e instalación de nueva cobertura con chapa/panel protegida con revestimiento HDX55 (55 µm) en ambas caras, con tornillería roscachapa galvanizada con arandela EPDM, remates perimetrales frontales con goterón y repercusión de plataformas elevadoras PEMP.</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D25" s="19" t="n">
         <v>533</v>
       </c>
-      <c r="E23" s="20" t="n">
+      <c r="E25" s="20" t="n">
         <v>95</v>
       </c>
-      <c r="F23" s="20">
-        <f>D23*E23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="F25" s="20">
+        <f>D25*E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Suministro e instalación de chapa grecada HDX55 en AMBAS CARAS en lado inferior de voladizos (cielo raso)
+Suministro e instalación de chapa grecada de acero estructural galvanizado con revestimiento anticorrosión marina Granite® HDX55 (55 µm) en AMBAS CARAS por la cara inferior de las viguetas en ménsula de los muelles de carga (cielo raso / forro inferior de voladizos). Incluye nivelación, fijación directa a viguetas mediante tornillería roscachapa de acero galvanizado con arandela vulcanizada de EPDM, perfilería perimetral de ajuste y remate, y repercusión completa de plataformas PEMP y fletes.</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="n">
+        <v>533.6</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>95</v>
+      </c>
+      <c r="F26" s="20">
+        <f>D26*E26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Suministro e instalación de chapa grecada HDX55 en AMBAS CARAS en tabica vertical de fachada sobre voladizos
+Suministro e instalación de chapa grecada de acero galvanizado con idéntico recubrimiento Granite® HDX55 (55 µm) en ambas caras en paramento vertical de tabica de fachada sobre marquesinas/voladizos de muelles. Incluye adaptaciones mecánicas en encuentros de peto, solapes estancos con cordón de butilo, tornillería roscachapa galvanizada con junta de estanqueidad de EPDM y medios de elevación con plataformas articuladas PEMP integrados.</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="n">
+        <v>186.5</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>95</v>
+      </c>
+      <c r="F27" s="20">
+        <f>D27*E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Rematería completa en acero con acabado HDX55, coronaciones, encuentros, mordidos y sellados
 Suministro, conformación en taller y montaje de 489,15 ml de rematería técnica plegada a medida (desarrollos 300-500 mm) en chapa de acero galvanizado con idéntico recubrimiento Granite® HDX55 (55 µm): 50,23 ml de cumbrera troquelada a dos aguas, 63,34 ml de remates laterales de hastial/testero con goterón, 30,22 ml de babero de coronación contra peto, 10,40 ml de remate de salto entre naves, 174,08 ml de goterones frontales y laterales de voladizo, 160,88 ml de baberos de encuentro voladizo-fachada y 10 unidades de mordidos y cajeados estancos en salidas de chimeneas y bajantes, fijados con tornillería galvanizada lacada con junta EPDM y doble sellado perimetral continuo con masilla hidro-expansiva de butilo y polímero elástico MS exterior.</t>
         </is>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>lote</t>
         </is>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D28" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E28" s="20" t="n">
         <v>14850</v>
       </c>
-      <c r="F24" s="20">
-        <f>D24*E24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="F28" s="20">
+        <f>D28*E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Seguridad y salud, protecciones colectivas en altura y protocolo aeroportuario AENA
 Implantación de medidas de seguridad y salud en altura bajo estricta normativa de AENA en terminal de carga: instalación de redes de seguridad anticaídas bajo faldones según norma UNE-EN 1263-1, líneas de vida provisionales homologadas UNE-EN 795, balizamiento perimetral de zonas de acopio y descarga, tramitación de Coordinación de Actividades Empresariales (CAE) en plataforma aeroportuaria, gestión de acreditaciones del personal y recursos preventivos permanentes en obra.</t>
         </is>
       </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>lote</t>
         </is>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D29" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="20" t="n">
+      <c r="E29" s="20" t="n">
         <v>9800</v>
       </c>
-      <c r="F25" s="20">
-        <f>D25*E25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="E26" s="21" t="inlineStr">
+      <c r="F29" s="20">
+        <f>D29*E29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>Subtotal Base Imponible (Obra Base):</t>
         </is>
       </c>
-      <c r="F26" s="22">
-        <f>SUM(F20:F25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="E27" s="23" t="inlineStr">
+      <c r="F30" s="22">
+        <f>SUM(F22:F29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" s="23" t="inlineStr">
         <is>
           <t>I.V.A. (21%) Obra Base:</t>
         </is>
       </c>
-      <c r="F27" s="24">
-        <f>F26*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="E28" s="25" t="inlineStr">
+      <c r="F31" s="24">
+        <f>F30*0.21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" s="25" t="inlineStr">
         <is>
           <t>TOTAL OBRA BASE (IVA incl.):</t>
         </is>
       </c>
-      <c r="F28" s="26">
-        <f>F26+F27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="F32" s="26">
+        <f>F30+F31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>PARTIDAS OPCIONALES INDEPENDIENTES (ACCESOS EN ACERO INOXIDABLE Y LÍNEA LUXTOP)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="27" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
         <is>
           <t>Partida</t>
         </is>
       </c>
-      <c r="B31" s="28" t="inlineStr">
+      <c r="B35" s="28" t="inlineStr">
         <is>
           <t>Concepto y Descripción Técnica</t>
         </is>
       </c>
-      <c r="C31" s="27" t="inlineStr">
+      <c r="C35" s="27" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D31" s="27" t="inlineStr">
+      <c r="D35" s="27" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E31" s="27" t="inlineStr">
+      <c r="E35" s="27" t="inlineStr">
         <is>
           <t>Precio Unitario (€)</t>
         </is>
       </c>
-      <c r="F31" s="27" t="inlineStr">
+      <c r="F35" s="27" t="inlineStr">
         <is>
           <t>Importe (€)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>OPC-01</t>
         </is>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>OPCIONAL 1: Escalera de gato con protección dorsal en acero inoxidable para acceso a voladizo (H ≈ 4,20 m)
 Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso seguro desde cota suelo a voladizo (altura aprox. 4,20 m, desarrollo total 5,30 m con desembarco). Incluye montantes verticales de pletina/tubo inox, peldaños antideslizantes estriados de seguridad, jaula de protección dorsal (crinolina) con aros y tirantes longitudinales en pletina inox a partir de 2,20 m, desembarco superior ensanchado con barandillas de salida de 1.100 mm, compuerta batiente de gravedad/muelle con cierre automático, placa de condena inferior anti-intrusión con candado en acero inoxidable para control de acceso aeroportuario AENA, y anclajes químicos estructurales en acero inox A4.</t>
         </is>
       </c>
-      <c r="C32" s="17" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>ud</t>
         </is>
       </c>
-      <c r="D32" s="19" t="n">
+      <c r="D36" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="20" t="n">
+      <c r="E36" s="20" t="n">
         <v>5005</v>
       </c>
-      <c r="F32" s="20">
-        <f>D32*E32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="F36" s="20">
+        <f>D36*E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>OPC-02</t>
         </is>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B37" s="18" t="inlineStr">
         <is>
           <t>OPCIONAL 2: Escalera de gato con protección dorsal en acero inoxidable para acceso a cubierta (H ≈ 6,80 m)
 Fabricación, suministro e instalación de escalera fija de gato según norma UNE-EN ISO 14122-4 realizada íntegramente en ACERO INOXIDABLE (AISI 304/316) para acceso técnico y de mantenimiento a la cubierta principal del edificio (altura aprox. 6,80 m, desarrollo total 7,90 m con desembarco). Incluye montantes de acero inox, peldaños antideslizantes mecanizados, jaula dorsal continua (crinolina) en acero inox a partir de 2,50 m de altura, desembarco superior protegido con barandillas de 1.100 mm y rodapié, puerta batiente de salida con resorte de cierre automático de seguridad, portón inferior abatible de bloqueo anti-intrusión con cerradura/candado de seguridad en acero inoxidable, y fijaciones estructurales en acero inoxidable A4.</t>
         </is>
       </c>
-      <c r="C33" s="17" t="inlineStr">
+      <c r="C37" s="17" t="inlineStr">
         <is>
           <t>ud</t>
         </is>
       </c>
-      <c r="D33" s="19" t="n">
+      <c r="D37" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="20" t="n">
+      <c r="E37" s="20" t="n">
         <v>7735</v>
       </c>
-      <c r="F33" s="20">
-        <f>D33*E33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="F37" s="20">
+        <f>D37*E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>OPC-03</t>
         </is>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B38" s="18" t="inlineStr">
         <is>
           <t>OPCIONAL 3: Línea de vida permanente homologada marca LUXTOP® s/ UNE-EN 795:2012 Tipo C sobre cubierta
 Suministro, replanteo, montaje y certificación oficial de sistema permanente de línea de vida horizontal continua de cable de acero inoxidable AISI 316 (Ø 8 mm) marca LUXTOP®, conforme a las normas UNE-EN 795:2012 Tipo C y CEN/TS 16415 (homologada para trabajo y rescate de hasta 4 operarios simultáneos). Instalación sobre cubierta de panel sándwich mediante postes terminales e intermedios con absorbedor de impacto dinámico patentado LuxTop®, bases de fijación estancas sobreelevadas con juntas de EPDM (evitando cualquier riesgo de filtración o puente térmico), tensor de cable con testigo micrométrico de tensión, pieza curva/esquina si procede, carros deslizadores pasantes transfronterizos sin necesidad de desconexión manual, placa de marcado identificativa CE, ensayos de tracción en obra y dossier de legalización con certificado visado.</t>
         </is>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="C38" s="17" t="inlineStr">
         <is>
           <t>ud</t>
         </is>
       </c>
-      <c r="D34" s="19" t="n">
+      <c r="D38" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="20" t="n">
+      <c r="E38" s="20" t="n">
         <v>18000</v>
       </c>
-      <c r="F34" s="20">
-        <f>D34*E34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="E35" s="29" t="inlineStr">
+      <c r="F38" s="20">
+        <f>D38*E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" s="29" t="inlineStr">
         <is>
           <t>Subtotal Opcionales (Base Imp.):</t>
         </is>
       </c>
-      <c r="F35" s="30">
-        <f>SUM(F32:F34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="E36" s="23" t="inlineStr">
+      <c r="F39" s="30">
+        <f>SUM(F36:F38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" s="23" t="inlineStr">
         <is>
           <t>I.V.A. (21%) Opcionales:</t>
         </is>
       </c>
-      <c r="F36" s="24">
-        <f>F35*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="E37" s="31" t="inlineStr">
+      <c r="F40" s="24">
+        <f>F39*0.21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" s="31" t="inlineStr">
         <is>
           <t>TOTAL OPCIONALES (IVA incl.):</t>
         </is>
       </c>
-      <c r="F37" s="32">
-        <f>F35+F36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="E39" s="33" t="inlineStr">
-        <is>
-          <t>TOTAL BASE IMPONIBLE CONJUNTA:</t>
-        </is>
-      </c>
-      <c r="F39" s="34">
-        <f>F26+F35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="E40" s="35" t="inlineStr">
-        <is>
-          <t>I.V.A. (21%) Conjunto:</t>
-        </is>
-      </c>
-      <c r="F40" s="36">
-        <f>F39*0.21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="E41" s="37" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL CONTRATO (IVA incl.):</t>
-        </is>
-      </c>
-      <c r="F41" s="38">
+      <c r="F41" s="32">
         <f>F39+F40</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>CONDICIONES COMERCIALES Y DE EJECUCIÓN</t>
-        </is>
+      <c r="E43" s="33" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL CONTRATO (BASE + OPCIONALES):</t>
+        </is>
+      </c>
+      <c r="F43" s="34">
+        <f>F30+F39</f>
+        <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>• Forma de pago:</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>A convenir con el cliente según avance y certificaciones de obra.</t>
-        </is>
+      <c r="E44" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL I.V.A. CONJUNTO (21%):</t>
+        </is>
+      </c>
+      <c r="F44" s="36">
+        <f>F43*0.21</f>
+        <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>• Plazo de ejecución:</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>2 a 3 meses desde la recepción de materiales en obra y formalización del contrato.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>• Garantías:</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>10 años en recubrimiento Granite® HDX55, en acero inoxidable y en sistema LuxTop®; 5 años en estanqueidad; 2 años en montaje</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>• Validez de oferta:</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>30 días naturales desde la fecha de emisión</t>
-        </is>
+      <c r="E45" s="37" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL FACTURA (IVA incl.):</t>
+        </is>
+      </c>
+      <c r="F45" s="38">
+        <f>F43+F44</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>